<commit_message>
bug fixes to new version
</commit_message>
<xml_diff>
--- a/templates.xlsx
+++ b/templates.xlsx
@@ -397,7 +397,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.75"/>
   <sheetData>
     <row r="1">
@@ -551,6 +551,18 @@
       <c r="R3" s="1" t="n"/>
       <c r="S3" s="1" t="n"/>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>first_name</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>